<commit_message>
Content and UI: record of soul hero, spirit medicine playlist, page copy sync
- Restore Record of Soul dark archival hero; merge terminology into archival note; timeline labels (footer brand / video catalog)
- Spirit Medicine: YouTube IDs from official playlist; display title stripping; workbook lead and titles
- Universal Matrix description (UMMA copy); about hero pills (下辖)
- Home: intro closing note accent; HomeProse closingNote
- site-preview.html and achievements report preview; scaffold and workbooks 01-07

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/01-首页.xlsx
+++ b/docs/page-copy/01-首页.xlsx
@@ -426,7 +426,7 @@
         <v>notes</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>home.achievements.card1Body</v>
       </c>
@@ -436,11 +436,17 @@
       <c r="C2" t="str">
         <v>paragraph / other</v>
       </c>
-      <c r="D2" t="str">
-        <v>255+ recorded public welfare live broadcasts; 800+ broadcast hours; TikTok pushed to 70,000+ highly relevant visitors; 1,200+ in-depth interviews; among them, in-depth communication with 400+ attached spirit ghosts. Helped 240+ patients with mental disorders quickly relieve the suffering caused by attached spirit ghosts on-site.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>255+有记录的公益直播；800+ 播出小时； Tiktok推送70,000+高相关人士来访 ；1,200+人次深度访谈；其中，与400+附体鬼魂深度交流。帮助240+精神障碍患者现场快速改善附体鬼魂带来的痛苦</v>
+      <c r="D2" t="str" xml:space="preserve">
+        <v xml:space="preserve">255+ recorded public welfare live broadcasts; 800+ broadcast hours; TikTok pushed to 70,000+ highly relevant visitors; 1,200+ in-depth interviews.
+Among them:
+In-depth communication with 400+ attached spirit ghosts.
+Helped 240+ patients with mental disorders quickly relieve the suffering caused by attached spirit ghosts on-site.</v>
+      </c>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">255+有记录的公益直播；800+ 播出小时； Tiktok推送70,000+高相关人士来访 ；1,200+人次深度访谈；
+其中：
+与 400+附体鬼魂深度交流。
+帮助 240+精神障碍患者现场快速改善附体鬼魂带来的痛苦</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -560,10 +566,10 @@
         <v>button / link</v>
       </c>
       <c r="D7" t="str">
-        <v>Continue to the full report.</v>
+        <v/>
       </c>
       <c r="E7" t="str">
-        <v>查看完整报告</v>
+        <v/>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -583,10 +589,10 @@
         <v>label</v>
       </c>
       <c r="D8" t="str">
-        <v>large-scale teamwork of many master members of SMSC</v>
+        <v>This is a masterpiece of large-scale global teamwork by the many master spirits of SMSC.</v>
       </c>
       <c r="E8" t="str">
-        <v>SMSC的众多高级掌控灵会员</v>
+        <v>这是 SMSC的众多高级掌控灵会员在全球大规模团队协作的杰作</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -606,10 +612,10 @@
         <v>label</v>
       </c>
       <c r="D9" t="str">
-        <v>masterpiece of global work</v>
+        <v/>
       </c>
       <c r="E9" t="str">
-        <v>全球大规模团队协作的杰作</v>
+        <v/>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -951,10 +957,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D24" t="str">
-        <v>In the physical world, the New Era of UMMA Organization has under its jurisdiction the Association of Spirit Realm's Ambassador (ASRA); members of ASRA are human beings in the physical world.In the spiritual world, the New Era of UMMA Organization has under its jurisdiction the Society of Master Spirit Controllers (SMSC); members of SMSC are senior master spirits in the spiritual world.This website is the official website of ASRA.The New Era of UMMA Organization and SMSC do not maintain any websites in the physical world.</v>
+        <v>In the physical world, the New Era of UMMA Organization has under its jurisdiction the Association of Spirit Realm's Ambassador (ASRA); members of ASRA are human beings in the physical world. ——In the spiritual world, the New Era of UMMA Organization has under its jurisdiction the Society of Master Spirit Controllers (SMSC); members of SMSC are senior master spirits in the spiritual world. **This website is the official website of ASRA.** The New Era of UMMA Organization and SMSC do not maintain any websites in the physical world.</v>
       </c>
       <c r="E24" t="str">
-        <v>——在现实世界， UMMA新世纪组织下辖灵魂世界使者协会（ASRA)；（ASRA)会员是现实世界的人类。在灵魂世界， UMMA新世纪组织下辖高级掌控灵协会( SMSC)；SMSC会员是灵魂世界的高级掌控灵。本网站是ASRA网站。UMMA新世纪组织和SMSC在现实世界没有网站</v>
+        <v>——在现实世界， UMMA新世纪组织下辖灵魂世界使者协会（ASRA)；（ASRA)会员是现实世界的人类。 ——在灵魂世界， UMMA新世纪组织下辖高级掌控灵协会( SMSC)；SMSC会员是灵魂世界的高级掌控灵。 **本网站是ASRA网站。** UMMA新世纪组织和SMSC在现实世界没有网站</v>
       </c>
       <c r="F24" t="str">
         <v/>
@@ -2350,7 +2356,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:G84"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
EN copy glossary overrides; InlineRich; About founders layout and photo; hero title wrap; page-copy sync
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/01-首页.xlsx
+++ b/docs/page-copy/01-首页.xlsx
@@ -635,10 +635,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D10" t="str">
-        <v>ASRA Founder Caros Wu will use PRCASG superpowers in 2025 to systematically communicate with the attached ghosts on American patients with mental disorders through TikTok live broadcasts, revealing the true living conditions of American ghosts, and quickly help patients in the live room improve various pains and disorders caused by the attached spirit ghosts.</v>
+        <v>ASRA Founder Caros Woo will use PRCASG superpowers in 2025 to systematically communicate with the attached ghosts on American patients with mental disorders through TikTok live broadcasts, revealing the true living conditions of American ghosts, and quickly help patients in the live room improve various pains and disorders caused by the attached spirit ghosts.</v>
       </c>
       <c r="E10" t="str">
-        <v>ASRA会长Caros吴在2025年使用PRCASG超能力通过TikTok直播系统性的与美国精神障碍患者身上的附体鬼魂系统性的交流美国鬼魂的真实生存状态，并且在直播间快速帮助患者改善附体鬼魂带来的各种病痛和灾害</v>
+        <v>ASRA会长Caros Woo在2025年使用PRCASG超能力通过TikTok直播系统性的与美国精神障碍患者身上的附体鬼魂系统性的交流美国鬼魂的真实生存状态，并且在直播间快速帮助患者改善附体鬼魂带来的各种病痛和灾害</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -946,7 +946,7 @@
         <v>Hero 文案在 home.*；导航在 nav.*</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" xml:space="preserve">
       <c r="A24" t="str">
         <v>home.intro.overviewAfter</v>
       </c>
@@ -956,8 +956,13 @@
       <c r="C24" t="str">
         <v>paragraph / other</v>
       </c>
-      <c r="D24" t="str">
-        <v>In the physical world, the New Era of UMMA Organization has under its jurisdiction the Association of Spirit Realm's Ambassador (ASRA); members of ASRA are human beings in the physical world. ——In the spiritual world, the New Era of UMMA Organization has under its jurisdiction the Society of Master Spirit Controllers (SMSC); members of SMSC are senior master spirits in the spiritual world. **This website is the official website of ASRA.** The New Era of UMMA Organization and SMSC do not maintain any websites in the physical world.</v>
+      <c r="D24" t="str" xml:space="preserve">
+        <v xml:space="preserve">In the physical world, the New Era of UMMA Organization has under its jurisdiction the Association of Spirit Realm's Ambassador (ASRA);
+Members of ASRA are human beings in the physical world. 
+——In the spiritual world, the New Era of UMMA Organization has under its jurisdiction the Society of Master Spirit Controllers (SMSC); 
+Members of SMSC are senior master spirits in the spiritual world. 
+**This website is the official website of ASRA.** 
+The New Era of UMMA Organization and SMSC do not maintain any websites in the physical world.</v>
       </c>
       <c r="E24" t="str">
         <v>——在现实世界， UMMA新世纪组织下辖灵魂世界使者协会（ASRA)；（ASRA)会员是现实世界的人类。 ——在灵魂世界， UMMA新世纪组织下辖高级掌控灵协会( SMSC)；SMSC会员是灵魂世界的高级掌控灵。 **本网站是ASRA网站。** UMMA新世纪组织和SMSC在现实世界没有网站</v>
@@ -1003,7 +1008,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D26" t="str">
-        <v>Spanning both the spiritual realm and the physical world</v>
+        <v>-----Spanning both the spiritual realm and the physical world</v>
       </c>
       <c r="E26" t="str">
         <v>跨越灵魂世界和现实世界的双领域组织</v>
@@ -1154,7 +1159,7 @@
         <v>Hero 文案在 home.*；导航在 nav.*</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" xml:space="preserve">
       <c r="A33" t="str">
         <v>home.intro.title</v>
       </c>
@@ -1164,8 +1169,9 @@
       <c r="C33" t="str">
         <v>heading</v>
       </c>
-      <c r="D33" t="str">
-        <v>What is The New Era of UMMA Organization?</v>
+      <c r="D33" t="str" xml:space="preserve">
+        <v xml:space="preserve">What is The New Era of 
+UMMA Organization?</v>
       </c>
       <c r="E33" t="str">
         <v>什么是 UMMA新世纪组织？</v>
@@ -1281,7 +1287,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D38" t="str">
-        <v>As the founder of ASRA, Woos family filmed a series of three-season documentaries of Woos ethereal life and world for over 1,400 minutes. This documentary is the first time in human history to systematically explore and reveal the truth of soul, life, world and governor with a large amount of evidence</v>
+        <v>As the founder of ASRA, Woos family filmed a series of three-season documentaries of Woos ethereal life and world for over 1,400 minutes. This documentary is the first time in human history to systematically explore and reveal the truth of spirit realm and governor with a large amount of evidence</v>
       </c>
       <c r="E38" t="str">
         <v>作为ASRA协会的会长和创始人，吴氏父子拍摄了超1400分钟《吴氏灵魂生命与世界》的3季系列纪录片。该纪录片是人类历史上第1次用大量的证据，系统性的探索和揭示了灵魂生命、世界和统御者的真相。</v>

</xml_diff>